<commit_message>
Auto-append .T suffix so Japanese codes can be entered as digits only
normalize_symbol() adds the Tokyo '.T' suffix when a symbol contains a
digit and has no suffix (e.g. 7203 -> 7203.T), while leaving US tickers
(AAPL) and already-suffixed codes untouched. Applied on both CSV and
Google Sheet loading. Template and README updated to reflect that '.T'
is optional.
</commit_message>
<xml_diff>
--- a/portfolio_template.xlsx
+++ b/portfolio_template.xlsx
@@ -242,7 +242,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>証券コード。日本株は末尾に .T を付けます（例: 7203.T）。米国株はティッカー（例: AAPL）。この列は必須です。</t>
+        <t>証券コード。日本株は数字だけでOK（例: 7203／末尾の .T は自動で付きます）。米国株はティッカー（例: AAPL）。この列は必須です。</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -606,7 +606,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>7203.T</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
@@ -624,7 +624,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>6758.T</t>
+          <t>6758</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -642,7 +642,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>9984.T</t>
+          <t>9984</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -854,7 +854,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>symbol（必須） … 証券コード。日本株は末尾に .T を付けます（例: 7203.T）。米国株はティッカー（例: AAPL）。</t>
+          <t>symbol（必須） … 証券コード。日本株は数字だけでOK（例: 7203）。末尾の .T は自動で付きます。米国株はティッカー（例: AAPL）。</t>
         </is>
       </c>
     </row>

</xml_diff>